<commit_message>
Add HR demo datasets for AI talent search
</commit_message>
<xml_diff>
--- a/web/data/members.xlsx
+++ b/web/data/members.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I93"/>
+  <dimension ref="A1:J93"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,6 +427,9 @@
       <c r="I1" t="str">
         <v>페르소나</v>
       </c>
+      <c r="J1" t="str">
+        <v>R/L 연차</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -456,6 +459,9 @@
       <c r="I2" t="str">
         <v>team_leader</v>
       </c>
+      <c r="J2">
+        <v>3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -485,6 +491,9 @@
       <c r="I3" t="str">
         <v>employee</v>
       </c>
+      <c r="J3">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -514,6 +523,9 @@
       <c r="I4" t="str">
         <v>employee</v>
       </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -543,6 +555,9 @@
       <c r="I5" t="str">
         <v>employee</v>
       </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -572,6 +587,9 @@
       <c r="I6" t="str">
         <v>employee</v>
       </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -601,6 +619,9 @@
       <c r="I7" t="str">
         <v>employee</v>
       </c>
+      <c r="J7">
+        <v>10</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -630,6 +651,9 @@
       <c r="I8" t="str">
         <v>employee</v>
       </c>
+      <c r="J8">
+        <v>8</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -659,6 +683,9 @@
       <c r="I9" t="str">
         <v>employee</v>
       </c>
+      <c r="J9">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -688,6 +715,9 @@
       <c r="I10" t="str">
         <v>employee</v>
       </c>
+      <c r="J10">
+        <v>2</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -717,6 +747,9 @@
       <c r="I11" t="str">
         <v>employee</v>
       </c>
+      <c r="J11">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -746,6 +779,9 @@
       <c r="I12" t="str">
         <v>employee</v>
       </c>
+      <c r="J12">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -775,6 +811,9 @@
       <c r="I13" t="str">
         <v>employee</v>
       </c>
+      <c r="J13">
+        <v>4</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -804,6 +843,9 @@
       <c r="I14" t="str">
         <v>employee</v>
       </c>
+      <c r="J14">
+        <v>3</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -833,6 +875,9 @@
       <c r="I15" t="str">
         <v>employee</v>
       </c>
+      <c r="J15">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -862,6 +907,9 @@
       <c r="I16" t="str">
         <v>team_leader</v>
       </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -891,6 +939,9 @@
       <c r="I17" t="str">
         <v>employee</v>
       </c>
+      <c r="J17">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -920,6 +971,9 @@
       <c r="I18" t="str">
         <v>employee</v>
       </c>
+      <c r="J18">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -949,6 +1003,9 @@
       <c r="I19" t="str">
         <v>employee</v>
       </c>
+      <c r="J19">
+        <v>4</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -978,6 +1035,9 @@
       <c r="I20" t="str">
         <v>employee</v>
       </c>
+      <c r="J20">
+        <v>5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1007,6 +1067,9 @@
       <c r="I21" t="str">
         <v>employee</v>
       </c>
+      <c r="J21">
+        <v>2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1036,6 +1099,9 @@
       <c r="I22" t="str">
         <v>employee</v>
       </c>
+      <c r="J22">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1065,6 +1131,9 @@
       <c r="I23" t="str">
         <v>employee</v>
       </c>
+      <c r="J23">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1094,6 +1163,9 @@
       <c r="I24" t="str">
         <v>employee</v>
       </c>
+      <c r="J24">
+        <v>3</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1123,6 +1195,9 @@
       <c r="I25" t="str">
         <v>employee</v>
       </c>
+      <c r="J25">
+        <v>7</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1152,6 +1227,9 @@
       <c r="I26" t="str">
         <v>employee</v>
       </c>
+      <c r="J26">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1181,6 +1259,9 @@
       <c r="I27" t="str">
         <v>employee</v>
       </c>
+      <c r="J27">
+        <v>2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1210,6 +1291,9 @@
       <c r="I28" t="str">
         <v>employee</v>
       </c>
+      <c r="J28">
+        <v>7</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1239,6 +1323,9 @@
       <c r="I29" t="str">
         <v>employee</v>
       </c>
+      <c r="J29">
+        <v>2</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1268,6 +1355,9 @@
       <c r="I30" t="str">
         <v>employee</v>
       </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1297,6 +1387,9 @@
       <c r="I31" t="str">
         <v>employee</v>
       </c>
+      <c r="J31">
+        <v>3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1326,6 +1419,9 @@
       <c r="I32" t="str">
         <v>employee</v>
       </c>
+      <c r="J32">
+        <v>7</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1355,6 +1451,9 @@
       <c r="I33" t="str">
         <v>employee</v>
       </c>
+      <c r="J33">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1384,6 +1483,9 @@
       <c r="I34" t="str">
         <v>calibration</v>
       </c>
+      <c r="J34">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1413,6 +1515,9 @@
       <c r="I35" t="str">
         <v>team_leader</v>
       </c>
+      <c r="J35">
+        <v>3</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1442,6 +1547,9 @@
       <c r="I36" t="str">
         <v>employee</v>
       </c>
+      <c r="J36">
+        <v>3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1471,6 +1579,9 @@
       <c r="I37" t="str">
         <v>employee</v>
       </c>
+      <c r="J37">
+        <v>6</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1500,6 +1611,9 @@
       <c r="I38" t="str">
         <v>employee</v>
       </c>
+      <c r="J38">
+        <v>9</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1529,6 +1643,9 @@
       <c r="I39" t="str">
         <v>employee</v>
       </c>
+      <c r="J39">
+        <v>8</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1558,6 +1675,9 @@
       <c r="I40" t="str">
         <v>employee</v>
       </c>
+      <c r="J40">
+        <v>3</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1587,6 +1707,9 @@
       <c r="I41" t="str">
         <v>employee</v>
       </c>
+      <c r="J41">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1616,13 +1739,16 @@
       <c r="I42" t="str">
         <v>employee</v>
       </c>
+      <c r="J42">
+        <v>9</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
         <v>G0043</v>
       </c>
       <c r="B43" t="str">
-        <v>남준민</v>
+        <v>김선재</v>
       </c>
       <c r="C43" t="str">
         <v>SK머티리얼즈</v>
@@ -1644,6 +1770,9 @@
       </c>
       <c r="I43" t="str">
         <v>employee</v>
+      </c>
+      <c r="J43">
+        <v>5</v>
       </c>
     </row>
     <row r="44">
@@ -1674,6 +1803,9 @@
       <c r="I44" t="str">
         <v>employee</v>
       </c>
+      <c r="J44">
+        <v>3</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -1703,6 +1835,9 @@
       <c r="I45" t="str">
         <v>employee</v>
       </c>
+      <c r="J45">
+        <v>4</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1732,6 +1867,9 @@
       <c r="I46" t="str">
         <v>employee</v>
       </c>
+      <c r="J46">
+        <v>5</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1761,6 +1899,9 @@
       <c r="I47" t="str">
         <v>employee</v>
       </c>
+      <c r="J47">
+        <v>9</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1790,6 +1931,9 @@
       <c r="I48" t="str">
         <v>employee</v>
       </c>
+      <c r="J48">
+        <v>2</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -1819,6 +1963,9 @@
       <c r="I49" t="str">
         <v>employee</v>
       </c>
+      <c r="J49">
+        <v>7</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1848,6 +1995,9 @@
       <c r="I50" t="str">
         <v>employee</v>
       </c>
+      <c r="J50">
+        <v>2</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -1877,6 +2027,9 @@
       <c r="I51" t="str">
         <v>employee</v>
       </c>
+      <c r="J51">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -1906,6 +2059,9 @@
       <c r="I52" t="str">
         <v>employee</v>
       </c>
+      <c r="J52">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -1935,6 +2091,9 @@
       <c r="I53" t="str">
         <v>executive</v>
       </c>
+      <c r="J53">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -1964,6 +2123,9 @@
       <c r="I54" t="str">
         <v>committee</v>
       </c>
+      <c r="J54">
+        <v>3</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -1993,6 +2155,9 @@
       <c r="I55" t="str">
         <v>team_leader</v>
       </c>
+      <c r="J55">
+        <v>3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2022,6 +2187,9 @@
       <c r="I56" t="str">
         <v>employee</v>
       </c>
+      <c r="J56">
+        <v>5</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2051,6 +2219,9 @@
       <c r="I57" t="str">
         <v>employee</v>
       </c>
+      <c r="J57">
+        <v>6</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2080,6 +2251,9 @@
       <c r="I58" t="str">
         <v>employee</v>
       </c>
+      <c r="J58">
+        <v>7</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2109,6 +2283,9 @@
       <c r="I59" t="str">
         <v>employee</v>
       </c>
+      <c r="J59">
+        <v>1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2138,6 +2315,9 @@
       <c r="I60" t="str">
         <v>employee</v>
       </c>
+      <c r="J60">
+        <v>7</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2167,6 +2347,9 @@
       <c r="I61" t="str">
         <v>employee</v>
       </c>
+      <c r="J61">
+        <v>4</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2196,6 +2379,9 @@
       <c r="I62" t="str">
         <v>employee</v>
       </c>
+      <c r="J62">
+        <v>7</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2225,6 +2411,9 @@
       <c r="I63" t="str">
         <v>employee</v>
       </c>
+      <c r="J63">
+        <v>10</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2254,6 +2443,9 @@
       <c r="I64" t="str">
         <v>employee</v>
       </c>
+      <c r="J64">
+        <v>3</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2283,6 +2475,9 @@
       <c r="I65" t="str">
         <v>employee</v>
       </c>
+      <c r="J65">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2312,6 +2507,9 @@
       <c r="I66" t="str">
         <v>employee</v>
       </c>
+      <c r="J66">
+        <v>10</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2341,6 +2539,9 @@
       <c r="I67" t="str">
         <v>employee</v>
       </c>
+      <c r="J67">
+        <v>4</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2370,6 +2571,9 @@
       <c r="I68" t="str">
         <v>employee</v>
       </c>
+      <c r="J68">
+        <v>3</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2399,6 +2603,9 @@
       <c r="I69" t="str">
         <v>employee</v>
       </c>
+      <c r="J69">
+        <v>4</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2428,6 +2635,9 @@
       <c r="I70" t="str">
         <v>employee</v>
       </c>
+      <c r="J70">
+        <v>2</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2457,6 +2667,9 @@
       <c r="I71" t="str">
         <v>employee</v>
       </c>
+      <c r="J71">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2486,6 +2699,9 @@
       <c r="I72" t="str">
         <v>employee</v>
       </c>
+      <c r="J72">
+        <v>4</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2515,6 +2731,9 @@
       <c r="I73" t="str">
         <v>employee</v>
       </c>
+      <c r="J73">
+        <v>9</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2544,6 +2763,9 @@
       <c r="I74" t="str">
         <v>employee</v>
       </c>
+      <c r="J74">
+        <v>3</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2573,6 +2795,9 @@
       <c r="I75" t="str">
         <v>team_leader</v>
       </c>
+      <c r="J75">
+        <v>3</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2602,6 +2827,9 @@
       <c r="I76" t="str">
         <v>employee</v>
       </c>
+      <c r="J76">
+        <v>5</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -2631,6 +2859,9 @@
       <c r="I77" t="str">
         <v>employee</v>
       </c>
+      <c r="J77">
+        <v>4</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -2660,6 +2891,9 @@
       <c r="I78" t="str">
         <v>employee</v>
       </c>
+      <c r="J78">
+        <v>5</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -2689,6 +2923,9 @@
       <c r="I79" t="str">
         <v>employee</v>
       </c>
+      <c r="J79">
+        <v>6</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -2718,13 +2955,16 @@
       <c r="I80" t="str">
         <v>employee</v>
       </c>
+      <c r="J80">
+        <v>1</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
         <v>EMP018</v>
       </c>
       <c r="B81" t="str">
-        <v>임수아</v>
+        <v>임가영</v>
       </c>
       <c r="C81" t="str">
         <v>SK머티리얼즈</v>
@@ -2746,6 +2986,9 @@
       </c>
       <c r="I81" t="str">
         <v>employee</v>
+      </c>
+      <c r="J81">
+        <v>3</v>
       </c>
     </row>
     <row r="82">
@@ -2776,6 +3019,9 @@
       <c r="I82" t="str">
         <v>employee</v>
       </c>
+      <c r="J82">
+        <v>1</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -2805,6 +3051,9 @@
       <c r="I83" t="str">
         <v>employee</v>
       </c>
+      <c r="J83">
+        <v>2</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -2834,6 +3083,9 @@
       <c r="I84" t="str">
         <v>employee</v>
       </c>
+      <c r="J84">
+        <v>3</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -2863,6 +3115,9 @@
       <c r="I85" t="str">
         <v>employee</v>
       </c>
+      <c r="J85">
+        <v>6</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -2892,6 +3147,9 @@
       <c r="I86" t="str">
         <v>employee</v>
       </c>
+      <c r="J86">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -2921,6 +3179,9 @@
       <c r="I87" t="str">
         <v>employee</v>
       </c>
+      <c r="J87">
+        <v>3</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -2950,6 +3211,9 @@
       <c r="I88" t="str">
         <v>employee</v>
       </c>
+      <c r="J88">
+        <v>1</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -2979,6 +3243,9 @@
       <c r="I89" t="str">
         <v>employee</v>
       </c>
+      <c r="J89">
+        <v>1</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -3008,6 +3275,9 @@
       <c r="I90" t="str">
         <v>employee</v>
       </c>
+      <c r="J90">
+        <v>3</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -3037,6 +3307,9 @@
       <c r="I91" t="str">
         <v>employee</v>
       </c>
+      <c r="J91">
+        <v>1</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -3066,6 +3339,9 @@
       <c r="I92" t="str">
         <v>employee</v>
       </c>
+      <c r="J92">
+        <v>2</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -3095,10 +3371,13 @@
       <c r="I93" t="str">
         <v>calibration</v>
       </c>
+      <c r="J93">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I93"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J93"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>